<commit_message>
updated turnouts and dashed lines
</commit_message>
<xml_diff>
--- a/data/config.xlsx
+++ b/data/config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\1-Projects\aewsd_frick_unit\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D204FF6-8195-4037-9CF1-6CDBB9B8C2F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C9AD673-72B4-43D9-8B83-2CC6A7EEDB57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3105" uniqueCount="1223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3113" uniqueCount="1229">
   <si>
     <t>Name</t>
   </si>
@@ -3624,9 +3624,6 @@
     <t>Proposed_Pipeline_20260119</t>
   </si>
   <si>
-    <t>G:\Arvin-Edison WSD-1215\121519005-DiGiorgio Unit\GIS\Feature\DiGiorgio_Unit\Proposed_pipeline_alt1_2024_0517.shp</t>
-  </si>
-  <si>
     <t>Existing Turnouts</t>
   </si>
   <si>
@@ -3654,61 +3651,82 @@
     <t>ASSE_NAME in ("North Canal Spreading Works","Sunset Spreading Works")</t>
   </si>
   <si>
+    <t>Phase_V2 == "2A Pipeline"</t>
+  </si>
+  <si>
+    <t>Phase != "1 Turnout"</t>
+  </si>
+  <si>
+    <t>Phase == "1 Turnout"</t>
+  </si>
+  <si>
+    <t>Desc_ == "Proposed"</t>
+  </si>
+  <si>
+    <t>Desc_ == "Existing"</t>
+  </si>
+  <si>
+    <t>ASSE_NAME</t>
+  </si>
+  <si>
+    <t>label_list</t>
+  </si>
+  <si>
+    <t>name, size_in</t>
+  </si>
+  <si>
+    <t>G:\Buena Vista WSD-1048\104814B1 DSIG App\GIS\Feature\AEWSD\Pipe.shp</t>
+  </si>
+  <si>
+    <t>Phase 1 Pipeline</t>
+  </si>
+  <si>
+    <t>#A3FF73</t>
+  </si>
+  <si>
+    <t>#FFFF73</t>
+  </si>
+  <si>
+    <t>#BFD9F2</t>
+  </si>
+  <si>
+    <t>C:\1-Projects\aewsd_frick_unit\data\clipped_usgs.parquet</t>
+  </si>
+  <si>
+    <t>Full USGS 10ft Ground Elevation</t>
+  </si>
+  <si>
+    <t>ContourEle</t>
+  </si>
+  <si>
+    <t>options</t>
+  </si>
+  <si>
+    <t>dashed</t>
+  </si>
+  <si>
+    <t>dashed_line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase_V2 in ("2B Pipeline", "3 Pipeline", "4 Pipeline", "5 Pipeline")			</t>
+  </si>
+  <si>
+    <t>APN_Lbl, Company_Name, Owner_Name, ASSE_NAME, ASSR_ACRES</t>
+  </si>
+  <si>
+    <t>\\EgnyteDrive\Clients\Arvin-Edison WSD-1215\121519005-DiGiorgio Unit\GIS\Feature\DiGiorgio_Unit\Proposed_pipeline_alt1_2024_0517.shp</t>
+  </si>
+  <si>
+    <t>\\EgnyteDrive\Clients\Arvin-Edison WSD-1215\121525005-DiGiorgio Unit Ph2b-5\400 GIS\Map\AEWSD_DiGiornio_Unit_Landowners\AEWSD_DiGiornio_Unit_Landowners.gdb</t>
+  </si>
+  <si>
+    <t>DiGiorgio_Unit_20260115</t>
+  </si>
+  <si>
+    <t>DiGiorgio Unit</t>
+  </si>
+  <si>
     <t>Type == "Alt 1"</t>
-  </si>
-  <si>
-    <t>Phase_V2 == "2A Pipeline"</t>
-  </si>
-  <si>
-    <t>Phase != "1 Turnout"</t>
-  </si>
-  <si>
-    <t>Phase == "1 Turnout"</t>
-  </si>
-  <si>
-    <t>Phase_V2 != "2A Pipeline"</t>
-  </si>
-  <si>
-    <t>Desc_ == "Proposed"</t>
-  </si>
-  <si>
-    <t>Desc_ == "Existing"</t>
-  </si>
-  <si>
-    <t>ASSE_NAME</t>
-  </si>
-  <si>
-    <t>label_list</t>
-  </si>
-  <si>
-    <t>name, size_in</t>
-  </si>
-  <si>
-    <t>G:\Buena Vista WSD-1048\104814B1 DSIG App\GIS\Feature\AEWSD\Pipe.shp</t>
-  </si>
-  <si>
-    <t>Phase 1 Pipeline</t>
-  </si>
-  <si>
-    <t>#A3FF73</t>
-  </si>
-  <si>
-    <t>#FFFF73</t>
-  </si>
-  <si>
-    <t>#BFD9F2</t>
-  </si>
-  <si>
-    <t>APN_1, Company_Name, Owner_Name, Total_Acreage</t>
-  </si>
-  <si>
-    <t>C:\1-Projects\aewsd_frick_unit\data\clipped_usgs.parquet</t>
-  </si>
-  <si>
-    <t>Full USGS 10ft Ground Elevation</t>
-  </si>
-  <si>
-    <t>ContourEle</t>
   </si>
 </sst>
 </file>
@@ -3795,7 +3813,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="25">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -3804,6 +3822,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -3883,32 +3904,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13AE2A8C-08DE-40F4-A2E7-494D02A4EEA7}" name="Table1" displayName="Table1" ref="A1:S46" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="A1:S46" xr:uid="{13AE2A8C-08DE-40F4-A2E7-494D02A4EEA7}"/>
-  <tableColumns count="19">
-    <tableColumn id="14" xr3:uid="{FD22FF16-AC11-4A88-BBBF-B095EEDCA4A7}" name="id" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{13AE2A8C-08DE-40F4-A2E7-494D02A4EEA7}" name="Table1" displayName="Table1" ref="A1:T47" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+  <autoFilter ref="A1:T47" xr:uid="{13AE2A8C-08DE-40F4-A2E7-494D02A4EEA7}"/>
+  <tableColumns count="20">
+    <tableColumn id="14" xr3:uid="{FD22FF16-AC11-4A88-BBBF-B095EEDCA4A7}" name="id" dataDxfId="22">
       <calculatedColumnFormula>COUNTA($B$2:B2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{ECDAEBCA-0BC9-4D6F-9D67-ED2F186EF0F7}" name="Name" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{750F9F45-74DA-4191-9FDD-C80D49E99883}" name="shape_type" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{DEA5C356-A0FC-4C8C-9968-5AC67FC3907E}" name="color" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{D15AE7DB-7AAD-471C-9773-F7621D0BAB27}" name="custom_icon" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{9FB5281E-350E-4B7D-9D58-0DB6B906BEBD}" name="size" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{D175D943-C463-43FC-9D90-342CE1DF7FBF}" name="alpha" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{2A7A5D16-0177-49A3-A357-AE17BC18B544}" name="label" dataDxfId="14"/>
-    <tableColumn id="16" xr3:uid="{A021074F-E293-4729-B760-95BDF80DC51A}" name="file_path" dataDxfId="13" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{ABE4042F-57EB-42CB-9347-7A941840A818}" name="file_type" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{ECDAEBCA-0BC9-4D6F-9D67-ED2F186EF0F7}" name="Name" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{750F9F45-74DA-4191-9FDD-C80D49E99883}" name="shape_type" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{DEA5C356-A0FC-4C8C-9968-5AC67FC3907E}" name="color" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{D15AE7DB-7AAD-471C-9773-F7621D0BAB27}" name="custom_icon" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{9FB5281E-350E-4B7D-9D58-0DB6B906BEBD}" name="size" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{D175D943-C463-43FC-9D90-342CE1DF7FBF}" name="alpha" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{2A7A5D16-0177-49A3-A357-AE17BC18B544}" name="label" dataDxfId="15"/>
+    <tableColumn id="16" xr3:uid="{A021074F-E293-4729-B760-95BDF80DC51A}" name="file_path" dataDxfId="14" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{ABE4042F-57EB-42CB-9347-7A941840A818}" name="file_type" dataDxfId="13">
       <calculatedColumnFormula>IF(AND(ISBLANK(K2),ISBLANK(L2)),"parquet",IF(ISBLANK(K2),"gdb","shp"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{FD57E4B2-F1EF-49AB-B319-5D04B985DCB6}" name="shp" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{C88AA5B1-0032-47EC-9D44-076891BB4F2B}" name="gdb" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{32F2F140-781D-475B-96FC-3B17A14657F3}" name="parquet" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{16B2C2C3-1747-4385-B461-84DE0EBE65B9}" name="layer" dataDxfId="8"/>
-    <tableColumn id="18" xr3:uid="{F571880E-2A58-4FC5-9051-AD39607E38B4}" name="filter" dataDxfId="7"/>
-    <tableColumn id="19" xr3:uid="{4ACDF9D3-EE1B-4D25-B520-3378B109EBB7}" name="label_list" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{70977AAF-43F2-425E-82FC-B3E65FBAA5F5}" name="clip_to_frick_x" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{19D89434-0A78-4277-B54E-50635DED3A14}" name="full" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{45E051C3-34F8-4959-9AE0-818EEF884C1A}" name="simple" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{FD57E4B2-F1EF-49AB-B319-5D04B985DCB6}" name="shp" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{C88AA5B1-0032-47EC-9D44-076891BB4F2B}" name="gdb" dataDxfId="11"/>
+    <tableColumn id="15" xr3:uid="{32F2F140-781D-475B-96FC-3B17A14657F3}" name="parquet" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{16B2C2C3-1747-4385-B461-84DE0EBE65B9}" name="layer" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{F571880E-2A58-4FC5-9051-AD39607E38B4}" name="filter" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{4ACDF9D3-EE1B-4D25-B520-3378B109EBB7}" name="label_list" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{70977AAF-43F2-425E-82FC-B3E65FBAA5F5}" name="clip_to_frick_x" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{19D89434-0A78-4277-B54E-50635DED3A14}" name="full" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{45E051C3-34F8-4959-9AE0-818EEF884C1A}" name="simple" dataDxfId="4"/>
+    <tableColumn id="20" xr3:uid="{EF425FD3-5E08-449B-99E2-86D7BEE4570A}" name="options" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4222,7 +4244,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U46"/>
+  <dimension ref="A1:U47"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="1" bestFit="1" customWidth="1"/>
@@ -4238,7 +4260,7 @@
     <col min="11" max="11" width="33.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="54.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="54.140625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="30.5703125" style="1" customWidth="1"/>
     <col min="15" max="15" width="60.42578125" style="1" customWidth="1"/>
     <col min="16" max="16" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.140625" style="1" bestFit="1" customWidth="1"/>
@@ -4298,7 +4320,7 @@
         <v>1190</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>1212</v>
+        <v>1209</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>1149</v>
@@ -4309,7 +4331,9 @@
       <c r="S1" s="1" t="s">
         <v>1142</v>
       </c>
-      <c r="T1" s="1"/>
+      <c r="T1" s="1" t="s">
+        <v>1219</v>
+      </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
@@ -5331,6 +5355,7 @@
       <c r="S28" s="1" t="b">
         <v>1</v>
       </c>
+      <c r="T28" s="1"/>
     </row>
     <row r="29" spans="1:20" ht="75" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
@@ -5362,6 +5387,7 @@
       <c r="K29" s="2" t="s">
         <v>1181</v>
       </c>
+      <c r="T29" s="1"/>
     </row>
     <row r="30" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -5396,6 +5422,7 @@
       <c r="K30" s="1" t="s">
         <v>1158</v>
       </c>
+      <c r="T30" s="1"/>
     </row>
     <row r="31" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -5427,6 +5454,7 @@
       <c r="K31" s="1" t="s">
         <v>1159</v>
       </c>
+      <c r="T31" s="1"/>
     </row>
     <row r="32" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -5461,14 +5489,15 @@
       <c r="K32" s="1" t="s">
         <v>1161</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="T32" s="1"/>
+    </row>
+    <row r="33" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <f>COUNTA($B$2:B33)</f>
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>1221</v>
+        <v>1217</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>33</v>
@@ -5492,20 +5521,21 @@
       <c r="K33" s="1" t="s">
         <v>1170</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="T33" s="1"/>
+    </row>
+    <row r="34" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <f>COUNTA($B$2:B34)</f>
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="F34" s="1">
         <v>2</v>
@@ -5527,22 +5557,23 @@
         <v>1171</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>1210</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>1207</v>
+      </c>
+      <c r="T34" s="1"/>
+    </row>
+    <row r="35" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <f>COUNTA($B$2:B35)</f>
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="F35" s="1">
         <v>2</v>
@@ -5564,10 +5595,11 @@
         <v>1171</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>1209</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>1206</v>
+      </c>
+      <c r="T35" s="1"/>
+    </row>
+    <row r="36" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <f>COUNTA($B$2:B36)</f>
         <v>35</v>
@@ -5600,8 +5632,9 @@
       <c r="K36" s="1" t="s">
         <v>1163</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="T36" s="1"/>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <f>COUNTA($B$2:B37)</f>
         <v>36</v>
@@ -5634,8 +5667,9 @@
       <c r="N37" s="1" t="s">
         <v>1166</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" ht="105" x14ac:dyDescent="0.25">
+      <c r="T37" s="1"/>
+    </row>
+    <row r="38" spans="1:20" ht="105" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <f>COUNTA($B$2:B38)</f>
         <v>37</v>
@@ -5672,16 +5706,17 @@
         <v>1186</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>1219</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>1223</v>
+      </c>
+      <c r="T38" s="1"/>
+    </row>
+    <row r="39" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <f>COUNTA($B$2:B39)</f>
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>24</v>
@@ -5690,7 +5725,7 @@
         <v>38</v>
       </c>
       <c r="F39" s="1">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G39" s="1">
         <v>1</v>
@@ -5709,19 +5744,20 @@
         <v>1192</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="P39" s="1" t="s">
         <v>1187</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="T39" s="1"/>
+    </row>
+    <row r="40" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <f>COUNTA($B$2:B40)</f>
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>24</v>
@@ -5730,7 +5766,7 @@
         <v>10</v>
       </c>
       <c r="F40" s="1">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G40" s="1">
         <v>1</v>
@@ -5749,19 +5785,20 @@
         <v>1192</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="P40" s="1" t="s">
         <v>1187</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="T40" s="1"/>
+    </row>
+    <row r="41" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <f>COUNTA($B$2:B41)</f>
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>33</v>
@@ -5789,13 +5826,14 @@
         <v>1193</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>1213</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>1210</v>
+      </c>
+      <c r="T41" s="1"/>
+    </row>
+    <row r="42" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <f>COUNTA($B$2:B42)</f>
         <v>41</v>
@@ -5829,22 +5867,23 @@
         <v>1193</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>1208</v>
+        <v>1222</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>1213</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+        <v>1210</v>
+      </c>
+      <c r="T42" s="1"/>
+    </row>
+    <row r="43" spans="1:20" ht="75" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <f>COUNTA($B$2:B43)</f>
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>33</v>
+        <v>1221</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>13</v>
@@ -5856,33 +5895,36 @@
         <v>1</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>1194</v>
+        <v>1224</v>
       </c>
       <c r="J43" s="1" t="str">
         <f t="shared" si="0"/>
         <v>shp</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>1194</v>
+        <v>1224</v>
       </c>
       <c r="L43" s="2"/>
       <c r="O43" s="1" t="s">
-        <v>1204</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>1228</v>
+      </c>
+      <c r="T43" s="1" t="s">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <f>COUNTA($B$2:B44)</f>
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="F44" s="1">
         <v>2</v>
@@ -5901,22 +5943,23 @@
         <v>1182</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="O44" s="1" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>1211</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>1208</v>
+      </c>
+      <c r="T44" s="1"/>
+    </row>
+    <row r="45" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <f>COUNTA($B$2:B45)</f>
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>33</v>
@@ -5931,17 +5974,18 @@
         <v>1</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>1214</v>
+        <v>1211</v>
       </c>
       <c r="J45" s="1" t="str">
         <f t="shared" si="0"/>
         <v>shp</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>1214</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>1211</v>
+      </c>
+      <c r="T45" s="1"/>
+    </row>
+    <row r="46" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <f>COUNTA($B$2:B46)</f>
         <v>45</v>
@@ -5962,21 +6006,57 @@
         <v>1</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>1222</v>
+        <v>1218</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>1220</v>
+        <v>1216</v>
       </c>
       <c r="J46" s="1" t="str">
         <f t="shared" si="0"/>
         <v>parquet</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>1220</v>
+        <v>1216</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>1222</v>
-      </c>
+        <v>1218</v>
+      </c>
+      <c r="T46" s="1"/>
+    </row>
+    <row r="47" spans="1:20" ht="60" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <f>COUNTA($B$2:B47)</f>
+        <v>46</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="1">
+        <v>10</v>
+      </c>
+      <c r="G47" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>1225</v>
+      </c>
+      <c r="J47" s="1" t="str">
+        <f>IF(AND(ISBLANK(K47),ISBLANK(L47)),"parquet",IF(ISBLANK(K47),"gdb","shp"))</f>
+        <v>gdb</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>1225</v>
+      </c>
+      <c r="N47" s="1" t="s">
+        <v>1226</v>
+      </c>
+      <c r="T47" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6696,9 +6776,12 @@
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B25" t="e">
+      <c r="A25">
+        <v>46</v>
+      </c>
+      <c r="B25" t="str">
         <f>_xlfn.XLOOKUP(simple5[[#This Row],[id]],Table1[id],Table1[Name])</f>
-        <v>#N/A</v>
+        <v>DiGiorgio Unit</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>